<commit_message>
Update World Cup 2026 stats 2026-09-12 20:18 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D172"/>
+  <dimension ref="A1:D173"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -3989,6 +3989,24 @@
         </is>
       </c>
     </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>2026-09-12T20:18:52+00:00</t>
+        </is>
+      </c>
+      <c r="B173" t="n">
+        <v>0</v>
+      </c>
+      <c r="C173" t="n">
+        <v>0</v>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-09-13 11:31 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D173"/>
+  <dimension ref="A1:D174"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -4007,6 +4007,24 @@
         </is>
       </c>
     </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>2026-09-13T11:31:13+00:00</t>
+        </is>
+      </c>
+      <c r="B174" t="n">
+        <v>0</v>
+      </c>
+      <c r="C174" t="n">
+        <v>0</v>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-09-13 20:28 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D174"/>
+  <dimension ref="A1:D175"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -4025,6 +4025,24 @@
         </is>
       </c>
     </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>2026-09-13T20:28:31+00:00</t>
+        </is>
+      </c>
+      <c r="B175" t="n">
+        <v>0</v>
+      </c>
+      <c r="C175" t="n">
+        <v>0</v>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-09-14 12:25 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D175"/>
+  <dimension ref="A1:D176"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -4043,6 +4043,24 @@
         </is>
       </c>
     </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>2026-09-14T12:25:15+00:00</t>
+        </is>
+      </c>
+      <c r="B176" t="n">
+        <v>0</v>
+      </c>
+      <c r="C176" t="n">
+        <v>0</v>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-09-14 21:36 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D176"/>
+  <dimension ref="A1:D177"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -4061,6 +4061,24 @@
         </is>
       </c>
     </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>2026-09-14T21:36:44+00:00</t>
+        </is>
+      </c>
+      <c r="B177" t="n">
+        <v>0</v>
+      </c>
+      <c r="C177" t="n">
+        <v>0</v>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-09-15 11:29 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D177"/>
+  <dimension ref="A1:D178"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -4079,6 +4079,24 @@
         </is>
       </c>
     </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>2026-09-15T11:29:58+00:00</t>
+        </is>
+      </c>
+      <c r="B178" t="n">
+        <v>0</v>
+      </c>
+      <c r="C178" t="n">
+        <v>0</v>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-09-15 20:58 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D178"/>
+  <dimension ref="A1:D179"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -4097,6 +4097,24 @@
         </is>
       </c>
     </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>2026-09-15T20:58:26+00:00</t>
+        </is>
+      </c>
+      <c r="B179" t="n">
+        <v>0</v>
+      </c>
+      <c r="C179" t="n">
+        <v>0</v>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-09-16 11:16 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D179"/>
+  <dimension ref="A1:D180"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -4115,6 +4115,24 @@
         </is>
       </c>
     </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>2026-09-16T11:16:07+00:00</t>
+        </is>
+      </c>
+      <c r="B180" t="n">
+        <v>0</v>
+      </c>
+      <c r="C180" t="n">
+        <v>0</v>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-09-16 21:00 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D180"/>
+  <dimension ref="A1:D181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -4133,6 +4133,24 @@
         </is>
       </c>
     </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>2026-09-16T21:00:11+00:00</t>
+        </is>
+      </c>
+      <c r="B181" t="n">
+        <v>0</v>
+      </c>
+      <c r="C181" t="n">
+        <v>0</v>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-09-17 11:24 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D181"/>
+  <dimension ref="A1:D182"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -4151,6 +4151,24 @@
         </is>
       </c>
     </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>2026-09-17T11:24:20+00:00</t>
+        </is>
+      </c>
+      <c r="B182" t="n">
+        <v>0</v>
+      </c>
+      <c r="C182" t="n">
+        <v>0</v>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-09-17 21:03 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D182"/>
+  <dimension ref="A1:D183"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -4169,6 +4169,24 @@
         </is>
       </c>
     </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>2026-09-17T21:03:06+00:00</t>
+        </is>
+      </c>
+      <c r="B183" t="n">
+        <v>0</v>
+      </c>
+      <c r="C183" t="n">
+        <v>0</v>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-09-18 10:57 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D183"/>
+  <dimension ref="A1:D184"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -4187,6 +4187,24 @@
         </is>
       </c>
     </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>2026-09-18T10:57:54+00:00</t>
+        </is>
+      </c>
+      <c r="B184" t="n">
+        <v>0</v>
+      </c>
+      <c r="C184" t="n">
+        <v>0</v>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-09-18 20:34 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D184"/>
+  <dimension ref="A1:D185"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -4205,6 +4205,24 @@
         </is>
       </c>
     </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>2026-09-18T20:34:47+00:00</t>
+        </is>
+      </c>
+      <c r="B185" t="n">
+        <v>0</v>
+      </c>
+      <c r="C185" t="n">
+        <v>0</v>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-09-19 10:41 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D185"/>
+  <dimension ref="A1:D186"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -4223,6 +4223,24 @@
         </is>
       </c>
     </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>2026-09-19T10:41:25+00:00</t>
+        </is>
+      </c>
+      <c r="B186" t="n">
+        <v>0</v>
+      </c>
+      <c r="C186" t="n">
+        <v>0</v>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-09-19 20:12 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D186"/>
+  <dimension ref="A1:D187"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -4241,6 +4241,24 @@
         </is>
       </c>
     </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>2026-09-19T20:12:25+00:00</t>
+        </is>
+      </c>
+      <c r="B187" t="n">
+        <v>0</v>
+      </c>
+      <c r="C187" t="n">
+        <v>0</v>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-09-20 11:03 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D187"/>
+  <dimension ref="A1:D188"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -4259,6 +4259,24 @@
         </is>
       </c>
     </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>2026-09-20T11:03:57+00:00</t>
+        </is>
+      </c>
+      <c r="B188" t="n">
+        <v>0</v>
+      </c>
+      <c r="C188" t="n">
+        <v>0</v>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-09-20 20:28 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D188"/>
+  <dimension ref="A1:D189"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -4277,6 +4277,24 @@
         </is>
       </c>
     </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>2026-09-20T20:28:48+00:00</t>
+        </is>
+      </c>
+      <c r="B189" t="n">
+        <v>0</v>
+      </c>
+      <c r="C189" t="n">
+        <v>0</v>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-09-21 12:31 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D189"/>
+  <dimension ref="A1:D190"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -4295,6 +4295,24 @@
         </is>
       </c>
     </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>2026-09-21T12:31:52+00:00</t>
+        </is>
+      </c>
+      <c r="B190" t="n">
+        <v>0</v>
+      </c>
+      <c r="C190" t="n">
+        <v>0</v>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-09-21 21:47 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D190"/>
+  <dimension ref="A1:D191"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -4313,6 +4313,24 @@
         </is>
       </c>
     </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>2026-09-21T21:47:29+00:00</t>
+        </is>
+      </c>
+      <c r="B191" t="n">
+        <v>0</v>
+      </c>
+      <c r="C191" t="n">
+        <v>0</v>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-09-22 11:20 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D191"/>
+  <dimension ref="A1:D192"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -4331,6 +4331,24 @@
         </is>
       </c>
     </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>2026-09-22T11:20:03+00:00</t>
+        </is>
+      </c>
+      <c r="B192" t="n">
+        <v>0</v>
+      </c>
+      <c r="C192" t="n">
+        <v>0</v>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-09-22 21:00 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D192"/>
+  <dimension ref="A1:D193"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -4349,6 +4349,24 @@
         </is>
       </c>
     </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>2026-09-22T21:00:05+00:00</t>
+        </is>
+      </c>
+      <c r="B193" t="n">
+        <v>0</v>
+      </c>
+      <c r="C193" t="n">
+        <v>0</v>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-09-23 11:14 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D193"/>
+  <dimension ref="A1:D194"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -4367,6 +4367,24 @@
         </is>
       </c>
     </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>2026-09-23T11:14:44+00:00</t>
+        </is>
+      </c>
+      <c r="B194" t="n">
+        <v>0</v>
+      </c>
+      <c r="C194" t="n">
+        <v>0</v>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-09-23 21:14 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D194"/>
+  <dimension ref="A1:D195"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -4385,6 +4385,24 @@
         </is>
       </c>
     </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>2026-09-23T21:14:51+00:00</t>
+        </is>
+      </c>
+      <c r="B195" t="n">
+        <v>0</v>
+      </c>
+      <c r="C195" t="n">
+        <v>0</v>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-09-24 11:29 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D195"/>
+  <dimension ref="A1:D196"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -4403,6 +4403,24 @@
         </is>
       </c>
     </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>2026-09-24T11:29:19+00:00</t>
+        </is>
+      </c>
+      <c r="B196" t="n">
+        <v>0</v>
+      </c>
+      <c r="C196" t="n">
+        <v>0</v>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-09-24 21:16 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D196"/>
+  <dimension ref="A1:D197"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -4421,6 +4421,24 @@
         </is>
       </c>
     </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>2026-09-24T21:16:19+00:00</t>
+        </is>
+      </c>
+      <c r="B197" t="n">
+        <v>0</v>
+      </c>
+      <c r="C197" t="n">
+        <v>0</v>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-09-25 11:35 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D197"/>
+  <dimension ref="A1:D198"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -4439,6 +4439,24 @@
         </is>
       </c>
     </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>2026-09-25T11:35:08+00:00</t>
+        </is>
+      </c>
+      <c r="B198" t="n">
+        <v>0</v>
+      </c>
+      <c r="C198" t="n">
+        <v>0</v>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-09-25 21:13 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D198"/>
+  <dimension ref="A1:D199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -4457,6 +4457,24 @@
         </is>
       </c>
     </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>2026-09-25T21:13:54+00:00</t>
+        </is>
+      </c>
+      <c r="B199" t="n">
+        <v>0</v>
+      </c>
+      <c r="C199" t="n">
+        <v>0</v>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-09-26 11:10 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D199"/>
+  <dimension ref="A1:D200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -4475,6 +4475,24 @@
         </is>
       </c>
     </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>2026-09-26T11:10:00+00:00</t>
+        </is>
+      </c>
+      <c r="B200" t="n">
+        <v>0</v>
+      </c>
+      <c r="C200" t="n">
+        <v>0</v>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-09-26 20:46 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D200"/>
+  <dimension ref="A1:D201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -4493,6 +4493,24 @@
         </is>
       </c>
     </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>2026-09-26T20:46:04+00:00</t>
+        </is>
+      </c>
+      <c r="B201" t="n">
+        <v>0</v>
+      </c>
+      <c r="C201" t="n">
+        <v>0</v>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-09-27 11:48 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D201"/>
+  <dimension ref="A1:D202"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -4511,6 +4511,24 @@
         </is>
       </c>
     </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>2026-09-27T11:48:14+00:00</t>
+        </is>
+      </c>
+      <c r="B202" t="n">
+        <v>0</v>
+      </c>
+      <c r="C202" t="n">
+        <v>0</v>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-09-27 21:02 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D202"/>
+  <dimension ref="A1:D203"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -4529,6 +4529,24 @@
         </is>
       </c>
     </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>2026-09-27T21:02:51+00:00</t>
+        </is>
+      </c>
+      <c r="B203" t="n">
+        <v>0</v>
+      </c>
+      <c r="C203" t="n">
+        <v>0</v>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-09-28 13:30 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D203"/>
+  <dimension ref="A1:D204"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -4547,6 +4547,24 @@
         </is>
       </c>
     </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>2026-09-28T13:30:38+00:00</t>
+        </is>
+      </c>
+      <c r="B204" t="n">
+        <v>0</v>
+      </c>
+      <c r="C204" t="n">
+        <v>0</v>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-09-28 23:01 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D204"/>
+  <dimension ref="A1:D205"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -4565,6 +4565,24 @@
         </is>
       </c>
     </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>2026-09-28T23:01:29+00:00</t>
+        </is>
+      </c>
+      <c r="B205" t="n">
+        <v>0</v>
+      </c>
+      <c r="C205" t="n">
+        <v>0</v>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-09-29 12:32 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D205"/>
+  <dimension ref="A1:D206"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -4583,6 +4583,24 @@
         </is>
       </c>
     </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>2026-09-29T12:32:38+00:00</t>
+        </is>
+      </c>
+      <c r="B206" t="n">
+        <v>0</v>
+      </c>
+      <c r="C206" t="n">
+        <v>0</v>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-09-29 21:59 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D206"/>
+  <dimension ref="A1:D207"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -4601,6 +4601,24 @@
         </is>
       </c>
     </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>2026-09-29T21:59:40+00:00</t>
+        </is>
+      </c>
+      <c r="B207" t="n">
+        <v>0</v>
+      </c>
+      <c r="C207" t="n">
+        <v>0</v>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-09-30 12:19 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D207"/>
+  <dimension ref="A1:D208"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -4619,6 +4619,24 @@
         </is>
       </c>
     </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>2026-09-30T12:19:47+00:00</t>
+        </is>
+      </c>
+      <c r="B208" t="n">
+        <v>0</v>
+      </c>
+      <c r="C208" t="n">
+        <v>0</v>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-09-30 21:58 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D208"/>
+  <dimension ref="A1:D209"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -4637,6 +4637,24 @@
         </is>
       </c>
     </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>2026-09-30T21:58:28+00:00</t>
+        </is>
+      </c>
+      <c r="B209" t="n">
+        <v>0</v>
+      </c>
+      <c r="C209" t="n">
+        <v>0</v>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-01 12:53 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D209"/>
+  <dimension ref="A1:D210"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -4655,6 +4655,24 @@
         </is>
       </c>
     </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>2026-10-01T12:53:18+00:00</t>
+        </is>
+      </c>
+      <c r="B210" t="n">
+        <v>0</v>
+      </c>
+      <c r="C210" t="n">
+        <v>0</v>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-01 22:26 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D210"/>
+  <dimension ref="A1:D211"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -4673,6 +4673,24 @@
         </is>
       </c>
     </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>2026-10-01T22:26:37+00:00</t>
+        </is>
+      </c>
+      <c r="B211" t="n">
+        <v>0</v>
+      </c>
+      <c r="C211" t="n">
+        <v>0</v>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-02 12:16 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D211"/>
+  <dimension ref="A1:D212"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -4691,6 +4691,24 @@
         </is>
       </c>
     </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>2026-10-02T12:16:16+00:00</t>
+        </is>
+      </c>
+      <c r="B212" t="n">
+        <v>0</v>
+      </c>
+      <c r="C212" t="n">
+        <v>0</v>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-02 21:56 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D212"/>
+  <dimension ref="A1:D213"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -4709,6 +4709,24 @@
         </is>
       </c>
     </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>2026-10-02T21:56:21+00:00</t>
+        </is>
+      </c>
+      <c r="B213" t="n">
+        <v>0</v>
+      </c>
+      <c r="C213" t="n">
+        <v>0</v>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-03 11:26 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D213"/>
+  <dimension ref="A1:D214"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -4727,6 +4727,24 @@
         </is>
       </c>
     </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>2026-10-03T11:26:37+00:00</t>
+        </is>
+      </c>
+      <c r="B214" t="n">
+        <v>0</v>
+      </c>
+      <c r="C214" t="n">
+        <v>0</v>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-03 20:43 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D214"/>
+  <dimension ref="A1:D215"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -4745,6 +4745,24 @@
         </is>
       </c>
     </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>2026-10-03T20:43:36+00:00</t>
+        </is>
+      </c>
+      <c r="B215" t="n">
+        <v>0</v>
+      </c>
+      <c r="C215" t="n">
+        <v>0</v>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-04 12:07 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D215"/>
+  <dimension ref="A1:D216"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -4763,6 +4763,24 @@
         </is>
       </c>
     </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>2026-10-04T12:07:46+00:00</t>
+        </is>
+      </c>
+      <c r="B216" t="n">
+        <v>0</v>
+      </c>
+      <c r="C216" t="n">
+        <v>0</v>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-04 20:59 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D216"/>
+  <dimension ref="A1:D217"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -4781,6 +4781,24 @@
         </is>
       </c>
     </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>2026-10-04T20:59:58+00:00</t>
+        </is>
+      </c>
+      <c r="B217" t="n">
+        <v>0</v>
+      </c>
+      <c r="C217" t="n">
+        <v>0</v>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-05 14:14 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D217"/>
+  <dimension ref="A1:D218"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -4799,6 +4799,24 @@
         </is>
       </c>
     </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>2026-10-05T14:14:09+00:00</t>
+        </is>
+      </c>
+      <c r="B218" t="n">
+        <v>0</v>
+      </c>
+      <c r="C218" t="n">
+        <v>0</v>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-05 23:50 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D218"/>
+  <dimension ref="A1:D219"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -4817,6 +4817,24 @@
         </is>
       </c>
     </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>2026-10-05T23:50:53+00:00</t>
+        </is>
+      </c>
+      <c r="B219" t="n">
+        <v>0</v>
+      </c>
+      <c r="C219" t="n">
+        <v>0</v>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-06 13:08 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D219"/>
+  <dimension ref="A1:D220"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -4835,6 +4835,24 @@
         </is>
       </c>
     </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>2026-10-06T13:08:50+00:00</t>
+        </is>
+      </c>
+      <c r="B220" t="n">
+        <v>0</v>
+      </c>
+      <c r="C220" t="n">
+        <v>0</v>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-06 22:27 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D220"/>
+  <dimension ref="A1:D221"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -4853,6 +4853,24 @@
         </is>
       </c>
     </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>2026-10-06T22:27:34+00:00</t>
+        </is>
+      </c>
+      <c r="B221" t="n">
+        <v>0</v>
+      </c>
+      <c r="C221" t="n">
+        <v>0</v>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-07 13:03 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D221"/>
+  <dimension ref="A1:D222"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -4871,6 +4871,24 @@
         </is>
       </c>
     </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>2026-10-07T13:03:52+00:00</t>
+        </is>
+      </c>
+      <c r="B222" t="n">
+        <v>0</v>
+      </c>
+      <c r="C222" t="n">
+        <v>0</v>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-07 22:51 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D222"/>
+  <dimension ref="A1:D223"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -4889,6 +4889,24 @@
         </is>
       </c>
     </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>2026-10-07T22:51:50+00:00</t>
+        </is>
+      </c>
+      <c r="B223" t="n">
+        <v>0</v>
+      </c>
+      <c r="C223" t="n">
+        <v>0</v>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-08 13:11 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D223"/>
+  <dimension ref="A1:D224"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -4907,6 +4907,24 @@
         </is>
       </c>
     </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>2026-10-08T13:11:18+00:00</t>
+        </is>
+      </c>
+      <c r="B224" t="n">
+        <v>0</v>
+      </c>
+      <c r="C224" t="n">
+        <v>0</v>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-08 23:03 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D224"/>
+  <dimension ref="A1:D225"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -4925,6 +4925,24 @@
         </is>
       </c>
     </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>2026-10-08T23:03:49+00:00</t>
+        </is>
+      </c>
+      <c r="B225" t="n">
+        <v>0</v>
+      </c>
+      <c r="C225" t="n">
+        <v>0</v>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-09 12:57 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D225"/>
+  <dimension ref="A1:D226"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -4943,6 +4943,24 @@
         </is>
       </c>
     </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>2026-10-09T12:57:39+00:00</t>
+        </is>
+      </c>
+      <c r="B226" t="n">
+        <v>0</v>
+      </c>
+      <c r="C226" t="n">
+        <v>0</v>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-09 22:23 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D226"/>
+  <dimension ref="A1:D227"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -4961,6 +4961,24 @@
         </is>
       </c>
     </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>2026-10-09T22:23:52+00:00</t>
+        </is>
+      </c>
+      <c r="B227" t="n">
+        <v>0</v>
+      </c>
+      <c r="C227" t="n">
+        <v>0</v>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-10 12:15 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D227"/>
+  <dimension ref="A1:D228"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -4979,6 +4979,24 @@
         </is>
       </c>
     </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>2026-10-10T12:15:12+00:00</t>
+        </is>
+      </c>
+      <c r="B228" t="n">
+        <v>0</v>
+      </c>
+      <c r="C228" t="n">
+        <v>0</v>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-10 21:18 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D228"/>
+  <dimension ref="A1:D229"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -4997,6 +4997,24 @@
         </is>
       </c>
     </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>2026-10-10T21:18:03+00:00</t>
+        </is>
+      </c>
+      <c r="B229" t="n">
+        <v>0</v>
+      </c>
+      <c r="C229" t="n">
+        <v>0</v>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-11 12:30 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D229"/>
+  <dimension ref="A1:D230"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -5015,6 +5015,24 @@
         </is>
       </c>
     </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>2026-10-11T12:30:32+00:00</t>
+        </is>
+      </c>
+      <c r="B230" t="n">
+        <v>0</v>
+      </c>
+      <c r="C230" t="n">
+        <v>0</v>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-11 21:37 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D230"/>
+  <dimension ref="A1:D231"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -5033,6 +5033,24 @@
         </is>
       </c>
     </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>2026-10-11T21:37:21+00:00</t>
+        </is>
+      </c>
+      <c r="B231" t="n">
+        <v>0</v>
+      </c>
+      <c r="C231" t="n">
+        <v>0</v>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-12 15:03 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D231"/>
+  <dimension ref="A1:D232"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -5051,6 +5051,24 @@
         </is>
       </c>
     </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>2026-10-12T15:03:00+00:00</t>
+        </is>
+      </c>
+      <c r="B232" t="n">
+        <v>0</v>
+      </c>
+      <c r="C232" t="n">
+        <v>0</v>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-13 00:17 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D232"/>
+  <dimension ref="A1:D233"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -5069,6 +5069,24 @@
         </is>
       </c>
     </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>2026-10-13T00:17:00+00:00</t>
+        </is>
+      </c>
+      <c r="B233" t="n">
+        <v>0</v>
+      </c>
+      <c r="C233" t="n">
+        <v>0</v>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-13 13:57 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D233"/>
+  <dimension ref="A1:D234"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -5087,6 +5087,24 @@
         </is>
       </c>
     </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>2026-10-13T13:57:13+00:00</t>
+        </is>
+      </c>
+      <c r="B234" t="n">
+        <v>0</v>
+      </c>
+      <c r="C234" t="n">
+        <v>0</v>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-13 22:23 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D234"/>
+  <dimension ref="A1:D235"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -5105,6 +5105,24 @@
         </is>
       </c>
     </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>2026-10-13T22:23:29+00:00</t>
+        </is>
+      </c>
+      <c r="B235" t="n">
+        <v>0</v>
+      </c>
+      <c r="C235" t="n">
+        <v>0</v>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-14 11:34 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D235"/>
+  <dimension ref="A1:D236"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -5123,6 +5123,24 @@
         </is>
       </c>
     </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>2026-10-14T11:34:14+00:00</t>
+        </is>
+      </c>
+      <c r="B236" t="n">
+        <v>0</v>
+      </c>
+      <c r="C236" t="n">
+        <v>0</v>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-14 21:21 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D236"/>
+  <dimension ref="A1:D237"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -5141,6 +5141,24 @@
         </is>
       </c>
     </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>2026-10-14T21:21:51+00:00</t>
+        </is>
+      </c>
+      <c r="B237" t="n">
+        <v>0</v>
+      </c>
+      <c r="C237" t="n">
+        <v>0</v>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-15 11:12 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D237"/>
+  <dimension ref="A1:D238"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -5159,6 +5159,24 @@
         </is>
       </c>
     </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>2026-10-15T11:12:42+00:00</t>
+        </is>
+      </c>
+      <c r="B238" t="n">
+        <v>0</v>
+      </c>
+      <c r="C238" t="n">
+        <v>0</v>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-15 21:02 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D238"/>
+  <dimension ref="A1:D239"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -5177,6 +5177,24 @@
         </is>
       </c>
     </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>2026-10-15T21:02:34+00:00</t>
+        </is>
+      </c>
+      <c r="B239" t="n">
+        <v>0</v>
+      </c>
+      <c r="C239" t="n">
+        <v>0</v>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-16 11:07 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D239"/>
+  <dimension ref="A1:D240"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -5195,6 +5195,24 @@
         </is>
       </c>
     </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>2026-10-16T11:07:39+00:00</t>
+        </is>
+      </c>
+      <c r="B240" t="n">
+        <v>0</v>
+      </c>
+      <c r="C240" t="n">
+        <v>0</v>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-16 20:37 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D240"/>
+  <dimension ref="A1:D241"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -5213,6 +5213,24 @@
         </is>
       </c>
     </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>2026-10-16T20:37:57+00:00</t>
+        </is>
+      </c>
+      <c r="B241" t="n">
+        <v>0</v>
+      </c>
+      <c r="C241" t="n">
+        <v>0</v>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-17 10:26 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D241"/>
+  <dimension ref="A1:D242"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -5231,6 +5231,24 @@
         </is>
       </c>
     </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>2026-10-17T10:26:53+00:00</t>
+        </is>
+      </c>
+      <c r="B242" t="n">
+        <v>0</v>
+      </c>
+      <c r="C242" t="n">
+        <v>0</v>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-17 20:16 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D242"/>
+  <dimension ref="A1:D243"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -5249,6 +5249,24 @@
         </is>
       </c>
     </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>2026-10-17T20:16:45+00:00</t>
+        </is>
+      </c>
+      <c r="B243" t="n">
+        <v>0</v>
+      </c>
+      <c r="C243" t="n">
+        <v>0</v>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-18 10:45 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D243"/>
+  <dimension ref="A1:D244"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -5267,6 +5267,24 @@
         </is>
       </c>
     </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>2026-10-18T10:45:33+00:00</t>
+        </is>
+      </c>
+      <c r="B244" t="n">
+        <v>0</v>
+      </c>
+      <c r="C244" t="n">
+        <v>0</v>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-18 20:15 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D244"/>
+  <dimension ref="A1:D245"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -5285,6 +5285,24 @@
         </is>
       </c>
     </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>2026-10-18T20:15:38+00:00</t>
+        </is>
+      </c>
+      <c r="B245" t="n">
+        <v>0</v>
+      </c>
+      <c r="C245" t="n">
+        <v>0</v>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-19 12:45 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D245"/>
+  <dimension ref="A1:D246"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -5303,6 +5303,24 @@
         </is>
       </c>
     </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>2026-10-19T12:45:59+00:00</t>
+        </is>
+      </c>
+      <c r="B246" t="n">
+        <v>0</v>
+      </c>
+      <c r="C246" t="n">
+        <v>0</v>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-19 22:05 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D246"/>
+  <dimension ref="A1:D247"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -5321,6 +5321,24 @@
         </is>
       </c>
     </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>2026-10-19T22:05:59+00:00</t>
+        </is>
+      </c>
+      <c r="B247" t="n">
+        <v>0</v>
+      </c>
+      <c r="C247" t="n">
+        <v>0</v>
+      </c>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-20 11:16 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D247"/>
+  <dimension ref="A1:D248"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -5339,6 +5339,24 @@
         </is>
       </c>
     </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>2026-10-20T11:16:25+00:00</t>
+        </is>
+      </c>
+      <c r="B248" t="n">
+        <v>0</v>
+      </c>
+      <c r="C248" t="n">
+        <v>0</v>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-20 21:21 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D248"/>
+  <dimension ref="A1:D249"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -5357,6 +5357,24 @@
         </is>
       </c>
     </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>2026-10-20T21:21:48+00:00</t>
+        </is>
+      </c>
+      <c r="B249" t="n">
+        <v>0</v>
+      </c>
+      <c r="C249" t="n">
+        <v>0</v>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-21 11:32 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D249"/>
+  <dimension ref="A1:D250"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -5375,6 +5375,24 @@
         </is>
       </c>
     </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>2026-10-21T11:32:21+00:00</t>
+        </is>
+      </c>
+      <c r="B250" t="n">
+        <v>0</v>
+      </c>
+      <c r="C250" t="n">
+        <v>0</v>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-21 21:22 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D250"/>
+  <dimension ref="A1:D251"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -5393,6 +5393,24 @@
         </is>
       </c>
     </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>2026-10-21T21:22:54+00:00</t>
+        </is>
+      </c>
+      <c r="B251" t="n">
+        <v>0</v>
+      </c>
+      <c r="C251" t="n">
+        <v>0</v>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-22 11:32 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D251"/>
+  <dimension ref="A1:D252"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -5411,6 +5411,24 @@
         </is>
       </c>
     </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>2026-10-22T11:32:34+00:00</t>
+        </is>
+      </c>
+      <c r="B252" t="n">
+        <v>0</v>
+      </c>
+      <c r="C252" t="n">
+        <v>0</v>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-22 21:18 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D252"/>
+  <dimension ref="A1:D253"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -5429,6 +5429,24 @@
         </is>
       </c>
     </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>2026-10-22T21:18:01+00:00</t>
+        </is>
+      </c>
+      <c r="B253" t="n">
+        <v>0</v>
+      </c>
+      <c r="C253" t="n">
+        <v>0</v>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-23 11:21 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D253"/>
+  <dimension ref="A1:D254"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -5447,6 +5447,24 @@
         </is>
       </c>
     </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>2026-10-23T11:21:45+00:00</t>
+        </is>
+      </c>
+      <c r="B254" t="n">
+        <v>0</v>
+      </c>
+      <c r="C254" t="n">
+        <v>0</v>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-23 21:07 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D254"/>
+  <dimension ref="A1:D255"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -5465,6 +5465,24 @@
         </is>
       </c>
     </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>2026-10-23T21:07:36+00:00</t>
+        </is>
+      </c>
+      <c r="B255" t="n">
+        <v>0</v>
+      </c>
+      <c r="C255" t="n">
+        <v>0</v>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-24 10:40 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D255"/>
+  <dimension ref="A1:D256"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -5483,6 +5483,24 @@
         </is>
       </c>
     </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>2026-10-24T10:40:55+00:00</t>
+        </is>
+      </c>
+      <c r="B256" t="n">
+        <v>0</v>
+      </c>
+      <c r="C256" t="n">
+        <v>0</v>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-24 20:24 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D256"/>
+  <dimension ref="A1:D257"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -5501,6 +5501,24 @@
         </is>
       </c>
     </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>2026-10-24T20:24:36+00:00</t>
+        </is>
+      </c>
+      <c r="B257" t="n">
+        <v>0</v>
+      </c>
+      <c r="C257" t="n">
+        <v>0</v>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-25 11:06 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D257"/>
+  <dimension ref="A1:D258"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -5519,6 +5519,24 @@
         </is>
       </c>
     </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>2026-10-25T11:06:02+00:00</t>
+        </is>
+      </c>
+      <c r="B258" t="n">
+        <v>0</v>
+      </c>
+      <c r="C258" t="n">
+        <v>0</v>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-25 20:31 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D258"/>
+  <dimension ref="A1:D259"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -5537,6 +5537,24 @@
         </is>
       </c>
     </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>2026-10-25T20:31:31+00:00</t>
+        </is>
+      </c>
+      <c r="B259" t="n">
+        <v>0</v>
+      </c>
+      <c r="C259" t="n">
+        <v>0</v>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-26 12:39 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D259"/>
+  <dimension ref="A1:D260"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -5555,6 +5555,24 @@
         </is>
       </c>
     </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>2026-10-26T12:39:17+00:00</t>
+        </is>
+      </c>
+      <c r="B260" t="n">
+        <v>0</v>
+      </c>
+      <c r="C260" t="n">
+        <v>0</v>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-26 22:24 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D260"/>
+  <dimension ref="A1:D261"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -5573,6 +5573,24 @@
         </is>
       </c>
     </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>2026-10-26T22:24:09+00:00</t>
+        </is>
+      </c>
+      <c r="B261" t="n">
+        <v>0</v>
+      </c>
+      <c r="C261" t="n">
+        <v>0</v>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-27 11:55 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D261"/>
+  <dimension ref="A1:D262"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -5591,6 +5591,24 @@
         </is>
       </c>
     </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>2026-10-27T11:55:08+00:00</t>
+        </is>
+      </c>
+      <c r="B262" t="n">
+        <v>0</v>
+      </c>
+      <c r="C262" t="n">
+        <v>0</v>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-27 21:54 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D262"/>
+  <dimension ref="A1:D263"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -5609,6 +5609,24 @@
         </is>
       </c>
     </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>2026-10-27T21:54:50+00:00</t>
+        </is>
+      </c>
+      <c r="B263" t="n">
+        <v>0</v>
+      </c>
+      <c r="C263" t="n">
+        <v>0</v>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-28 12:32 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D263"/>
+  <dimension ref="A1:D264"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -5627,6 +5627,24 @@
         </is>
       </c>
     </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>2026-10-28T12:32:20+00:00</t>
+        </is>
+      </c>
+      <c r="B264" t="n">
+        <v>0</v>
+      </c>
+      <c r="C264" t="n">
+        <v>0</v>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-28 22:18 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D264"/>
+  <dimension ref="A1:D265"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -5645,6 +5645,24 @@
         </is>
       </c>
     </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>2026-10-28T22:18:53+00:00</t>
+        </is>
+      </c>
+      <c r="B265" t="n">
+        <v>0</v>
+      </c>
+      <c r="C265" t="n">
+        <v>0</v>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-29 12:42 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D265"/>
+  <dimension ref="A1:D266"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -5663,6 +5663,24 @@
         </is>
       </c>
     </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>2026-10-29T12:42:39+00:00</t>
+        </is>
+      </c>
+      <c r="B266" t="n">
+        <v>0</v>
+      </c>
+      <c r="C266" t="n">
+        <v>0</v>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-29 22:32 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D266"/>
+  <dimension ref="A1:D267"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -5681,6 +5681,24 @@
         </is>
       </c>
     </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>2026-10-29T22:32:06+00:00</t>
+        </is>
+      </c>
+      <c r="B267" t="n">
+        <v>0</v>
+      </c>
+      <c r="C267" t="n">
+        <v>0</v>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-30 12:34 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D267"/>
+  <dimension ref="A1:D268"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -5699,6 +5699,24 @@
         </is>
       </c>
     </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>2026-10-30T12:34:20+00:00</t>
+        </is>
+      </c>
+      <c r="B268" t="n">
+        <v>0</v>
+      </c>
+      <c r="C268" t="n">
+        <v>0</v>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-30 22:01 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D268"/>
+  <dimension ref="A1:D269"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -5717,6 +5717,24 @@
         </is>
       </c>
     </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>2026-10-30T22:01:07+00:00</t>
+        </is>
+      </c>
+      <c r="B269" t="n">
+        <v>0</v>
+      </c>
+      <c r="C269" t="n">
+        <v>0</v>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-31 11:59 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D269"/>
+  <dimension ref="A1:D270"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -5735,6 +5735,24 @@
         </is>
       </c>
     </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>2026-10-31T11:59:58+00:00</t>
+        </is>
+      </c>
+      <c r="B270" t="n">
+        <v>0</v>
+      </c>
+      <c r="C270" t="n">
+        <v>0</v>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update World Cup 2026 stats 2026-10-31 21:09 UTC
</commit_message>
<xml_diff>
--- a/data/world_cup_2026.xlsx
+++ b/data/world_cup_2026.xlsx
@@ -880,7 +880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D270"/>
+  <dimension ref="A1:D271"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -5753,6 +5753,24 @@
         </is>
       </c>
     </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>2026-10-31T21:09:34+00:00</t>
+        </is>
+      </c>
+      <c r="B271" t="n">
+        <v>0</v>
+      </c>
+      <c r="C271" t="n">
+        <v>0</v>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>